<commit_message>
SPM-32: fixed typo in test cases review
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-32_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-32_Test_Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janelleip/Documents/GitHub/IS212/docs/test-cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{637C4577-138A-D84A-BC97-576CD62C8714}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09421603-A104-D045-A9DB-C8A5F5451349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -835,15 +835,15 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1079,16 +1079,16 @@
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="19"/>
     </row>
     <row r="3" spans="1:9" ht="14" x14ac:dyDescent="0.15">
       <c r="A3" s="7" t="s">
@@ -1423,116 +1423,117 @@
       <c r="A18" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="19" t="s">
+      <c r="C18" s="18"/>
+      <c r="D18" s="19"/>
+      <c r="E18" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="F18" s="18"/>
+      <c r="F18" s="19"/>
     </row>
     <row r="19" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="16" t="s">
+      <c r="B19" s="20" t="s">
         <v>64</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="16" t="s">
+      <c r="C19" s="18"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="F19" s="18"/>
+      <c r="F19" s="19"/>
     </row>
     <row r="20" spans="1:6" ht="112" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="16" t="s">
+      <c r="B20" s="20" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="16" t="s">
+      <c r="C20" s="18"/>
+      <c r="D20" s="19"/>
+      <c r="E20" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="F20" s="18"/>
+      <c r="F20" s="19"/>
     </row>
     <row r="21" spans="1:6" ht="98.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="16" t="s">
+      <c r="B21" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="16" t="s">
+      <c r="C21" s="18"/>
+      <c r="D21" s="19"/>
+      <c r="E21" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="F21" s="18"/>
+      <c r="F21" s="19"/>
     </row>
     <row r="22" spans="1:6" ht="58" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B22" s="16" t="s">
+      <c r="B22" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="18"/>
-      <c r="E22" s="16" t="s">
+      <c r="C22" s="18"/>
+      <c r="D22" s="19"/>
+      <c r="E22" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="F22" s="18"/>
+      <c r="F22" s="19"/>
     </row>
     <row r="23" spans="1:6" ht="44.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="16" t="s">
+      <c r="B23" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="C23" s="17"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="16" t="s">
+      <c r="C23" s="18"/>
+      <c r="D23" s="19"/>
+      <c r="E23" s="20" t="s">
         <v>44</v>
       </c>
-      <c r="F23" s="18"/>
+      <c r="F23" s="19"/>
     </row>
     <row r="24" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B24" s="16" t="s">
+      <c r="B24" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="C24" s="17"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="16" t="s">
+      <c r="C24" s="18"/>
+      <c r="D24" s="19"/>
+      <c r="E24" s="20" t="s">
         <v>78</v>
       </c>
-      <c r="F24" s="18"/>
+      <c r="F24" s="19"/>
     </row>
     <row r="25" spans="1:6" ht="31" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="16" t="s">
+      <c r="B25" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="C25" s="17"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="16" t="s">
+      <c r="C25" s="18"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="F25" s="18"/>
+      <c r="F25" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="B22:D22"/>
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B20:D20"/>
@@ -1549,7 +1550,6 @@
     <mergeCell ref="E21:F21"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="E24:F24"/>
-    <mergeCell ref="B22:D22"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'TC01'!A1" display="TC01" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -1717,7 +1717,7 @@
       <c r="A21" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="16" t="s">
         <v>151</v>
       </c>
     </row>
@@ -2317,7 +2317,7 @@
         <v>109</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>174</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>

<commit_message>
SPM-32: updated commit date for test cases
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-32_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-32_Test_Cases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/janelleip/Documents/GitHub/IS212/docs/test-cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09421603-A104-D045-A9DB-C8A5F5451349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54DBF605-C2D5-3442-AAD1-9100765366C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15980" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" r:id="rId1"/>
@@ -651,7 +651,7 @@
 Step 6: The request for 'SPM32 Advisers Workshop' is still listed as 'Pending'.</t>
   </si>
   <si>
-    <t>8b8833c</t>
+    <t>f707184</t>
   </si>
 </sst>
 </file>
@@ -838,12 +838,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1079,7 +1079,7 @@
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="B1" s="20" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="18"/>
@@ -1423,12 +1423,12 @@
       <c r="A18" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="17" t="s">
+      <c r="B18" s="20" t="s">
         <v>62</v>
       </c>
       <c r="C18" s="18"/>
       <c r="D18" s="19"/>
-      <c r="E18" s="17" t="s">
+      <c r="E18" s="20" t="s">
         <v>63</v>
       </c>
       <c r="F18" s="19"/>
@@ -1437,12 +1437,12 @@
       <c r="A19" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="17" t="s">
         <v>64</v>
       </c>
       <c r="C19" s="18"/>
       <c r="D19" s="19"/>
-      <c r="E19" s="20" t="s">
+      <c r="E19" s="17" t="s">
         <v>65</v>
       </c>
       <c r="F19" s="19"/>
@@ -1451,12 +1451,12 @@
       <c r="A20" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="17" t="s">
         <v>66</v>
       </c>
       <c r="C20" s="18"/>
       <c r="D20" s="19"/>
-      <c r="E20" s="20" t="s">
+      <c r="E20" s="17" t="s">
         <v>67</v>
       </c>
       <c r="F20" s="19"/>
@@ -1465,12 +1465,12 @@
       <c r="A21" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="17" t="s">
         <v>69</v>
       </c>
       <c r="C21" s="18"/>
       <c r="D21" s="19"/>
-      <c r="E21" s="20" t="s">
+      <c r="E21" s="17" t="s">
         <v>70</v>
       </c>
       <c r="F21" s="19"/>
@@ -1479,12 +1479,12 @@
       <c r="A22" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="17" t="s">
         <v>72</v>
       </c>
       <c r="C22" s="18"/>
       <c r="D22" s="19"/>
-      <c r="E22" s="20" t="s">
+      <c r="E22" s="17" t="s">
         <v>73</v>
       </c>
       <c r="F22" s="19"/>
@@ -1493,12 +1493,12 @@
       <c r="A23" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="17" t="s">
         <v>75</v>
       </c>
       <c r="C23" s="18"/>
       <c r="D23" s="19"/>
-      <c r="E23" s="20" t="s">
+      <c r="E23" s="17" t="s">
         <v>44</v>
       </c>
       <c r="F23" s="19"/>
@@ -1507,12 +1507,12 @@
       <c r="A24" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B24" s="20" t="s">
+      <c r="B24" s="17" t="s">
         <v>77</v>
       </c>
       <c r="C24" s="18"/>
       <c r="D24" s="19"/>
-      <c r="E24" s="20" t="s">
+      <c r="E24" s="17" t="s">
         <v>78</v>
       </c>
       <c r="F24" s="19"/>
@@ -1521,18 +1521,19 @@
       <c r="A25" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="17" t="s">
         <v>79</v>
       </c>
       <c r="C25" s="18"/>
       <c r="D25" s="19"/>
-      <c r="E25" s="20" t="s">
+      <c r="E25" s="17" t="s">
         <v>80</v>
       </c>
       <c r="F25" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="E24:F24"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="B24:D24"/>
@@ -1549,7 +1550,6 @@
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="E21:F21"/>
     <mergeCell ref="B23:D23"/>
-    <mergeCell ref="E24:F24"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'TC01'!A1" display="TC01" xr:uid="{00000000-0004-0000-0000-000000000000}"/>

</xml_diff>

<commit_message>
docs/regression sprint 4 generation
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-32_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-32_Test_Cases.xlsx
@@ -31,7 +31,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -83,6 +83,13 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color theme="1"/>
+      <sz val="10"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -109,7 +116,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -191,11 +198,44 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -242,6 +282,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,6 +597,7 @@
       <c r="H1" s="18" t="n"/>
       <c r="I1" s="19" t="n"/>
     </row>
+    <row r="2"/>
     <row r="3" ht="14" customHeight="1">
       <c r="A3" s="20" t="inlineStr">
         <is>
@@ -672,11 +717,15 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="H5" s="17" t="n"/>
-      <c r="I5" s="17" t="n"/>
+      <c r="I5" s="17" t="inlineStr">
+        <is>
+          <t>#129 (Week 7 #5)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="42" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -1072,6 +1121,8 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18" ht="14" customHeight="1">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -1256,13 +1307,13 @@
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B23:D23"/>
     <mergeCell ref="E19:F19"/>
-    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="E18:F18"/>
     <mergeCell ref="B20:D20"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="B25:D25"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="E21:F21"/>
   </mergeCells>
@@ -1487,6 +1538,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -1769,6 +1822,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -2056,6 +2110,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -2340,6 +2396,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -3056,6 +3114,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -3145,64 +3205,72 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="24.83203125" customWidth="1" min="1" max="1"/>
     <col width="56.83203125" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="13" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="54" customHeight="1">
+      <c r="A1" s="22" t="inlineStr">
+        <is>
+          <t>v2 (2026-10-30): The Event Operations Manager is now shown as the 'Event Coordinator Lead' (SPM-84 AC1, forum #129, Week 7 Change #5) - the same role, accounts, permissions and pages. Read 'Ops Manager' in this case as 'Event Coordinator Lead'; the steps and everything else are unchanged.</t>
+        </is>
+      </c>
+      <c r="B1" s="23" t="n"/>
+    </row>
+    <row r="2" ht="13" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="2" t="n"/>
-    </row>
-    <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="17.5" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>SPM-32-TC02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="B3" s="11" t="inlineStr">
-        <is>
-          <t>Only the assigned coordinator is offered Review on a pending change request - not another coordinator or the organiser who raised it</t>
         </is>
       </c>
     </row>
     <row r="4" ht="44.5" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B4" s="11" t="inlineStr">
+        <is>
+          <t>Only the assigned coordinator is offered Review on a pending change request - not another coordinator or the organiser who raised it</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>npm run fixtures:spm32 has been run. 'SPM32 Harbour Briefing' (coordinator Daniel Tan, organiser Rachel Ng) has a pending change request. Nothing is saved in this case.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="112" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+    <row r="6" ht="112" customHeight="1">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>1. Log in as priya.raj@connectsphere.com / password123
 2. Click 'Change Requests' in the sidebar
@@ -3212,13 +3280,13 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="44.5" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+    <row r="7" ht="44.5" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Event: SPM32 Harbour Briefing (coordinator Daniel Tan)
 Other coordinator: Priya Raj
@@ -3226,13 +3294,13 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="98.5" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="8" ht="98.5" customHeight="1">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Step 2: The page lists the request for 'SPM32 Other Coordinator Forum' and none of Daniel Tan's SPM32 events.
 Step 3: The event opens with no 'Change requests' card: only the event's organisers, its assigned coordinator and the Ops Manager see its change requests (SPM-35).
@@ -3240,123 +3308,125 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="9" ht="17.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="13" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="10" ht="13" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B10" s="12" t="n">
         <v>46320</v>
       </c>
     </row>
-    <row r="10" ht="13" customHeight="1"/>
-    <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="11" ht="13" customHeight="1"/>
+    <row r="12" ht="13" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="6" t="n"/>
-    </row>
-    <row r="12" ht="71.5" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="71.5" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>Priya Raj's Change Requests page listed SPM32 Other Coordinator Forum and none of Daniel Tan's events. Opening SPM32 Harbour Briefing as Priya showed no 'Change requests' card. As Rachel Ng the card listed the request as 'Pending' with no 'Review' link.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="17.5" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="14" ht="17.5" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="44.5" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15" ht="44.5" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Step 3 first expected the card with no Review link; another coordinator is not shown the card at all (SPM-35), so the expected result was corrected before this run.</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="17.5" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16" ht="17.5" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B17" s="15" t="n">
         <v>46320</v>
       </c>
     </row>
-    <row r="17" ht="17.5" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+    <row r="18" ht="17.5" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Commit</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>8d8aa0d</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="19"/>
+    <row r="20" ht="15.75" customHeight="1"/>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B20" s="5" t="n"/>
-    </row>
-    <row r="21" ht="92" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="B21" s="5" t="n"/>
+    </row>
+    <row r="22" ht="92" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>Step 2: The page lists the request for 'SPM32 Other Coordinator Forum' and none of Daniel Tan's SPM32 events.
 Step 3: The event opens with no 'Change requests' card: only the event's organisers, its assigned coordinator and the Ops Manager see its change requests (SPM-35).
@@ -3364,65 +3434,68 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="71" customHeight="1">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="24" ht="71" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B23" s="13" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>NA</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>Janelle</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>Date of Execution</t>
-        </is>
-      </c>
-      <c r="B25" s="15" t="n">
-        <v>46322</v>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>Janelle</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n">
+        <v>46322</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
           <t>Commit</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>f707184</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3633,6 +3706,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -3915,6 +3990,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="15.75" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
@@ -4202,6 +4278,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -4491,6 +4569,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -4780,6 +4860,8 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
+    <row r="19"/>
     <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>

</xml_diff>